<commit_message>
Tab B doc refreshes: PRD amendments tab (5 rows incl provider-on-hold), UX doc rows (SnapTrade truth, menu, FAB), design-doc retroactive+refresh rows, flows v2
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-PRD-v1.1-2026-07-01.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-PRD-v1.1-2026-07-01.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Calculation catalog" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Sameness contract" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="NFR · data integrity · Plaid" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Amendments v1.1→v1.2" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Acceptance criteria'!$A$1:$D$171</definedName>
@@ -834,6 +835,158 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" style="24" min="1" max="1"/>
+    <col width="30" customWidth="1" style="24" min="2" max="2"/>
+    <col width="95" customWidth="1" style="24" min="3" max="3"/>
+    <col width="40" customWidth="1" style="24" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>New/changed acceptance criteria</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Why</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>F2 Debt — repayment shapes</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Debt.payment_type ∈ installment | revolving | due_in_full, USER-EDITABLE via the one DebtEditorSheet ("How is it repaid?"). Installment: real payment ↔ paid-off-by, either computed (monthsToClear/paymentToClearBy); saves min=payment. Due-in-full: amount+date → ONE dated big-ticket in the grid + bill calendar + Later; zero monthly obligation in DTI/cash flow; balance still in net worth; payoffPlan clears it in its due month. Deferred loans: first_payment_date captured in the installment shape ("Payments start").</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Founder-approved 2026-07-31 (mock debt-editor-v1); B47 finding 11</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>F6/F9 Big one-time costs</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>NEW: bigCosts[] {label, amount(today $), year} captured on /big-costs; simulate() subtracts each, inflated to its year, accumulation AND decumulation; the capture screen states the odds delta via the SAME selector; empty state = "odds assume none". Hub row "What big costs are coming?" both lenses.</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Founder-approved 2026-08-01/02 (mock big-costs-v1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>F11 Plan hub — dynamic door + next decision</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>First-day door counts ONLY missing answers (age/spend/have) and credits live accounts ("already in: N connected accounts, $X counted"). ONE dated next-decision card: RMD-due-untaken outranks SS-window; absent when nothing due. RULE SOURCE: nextDecision (domain/planning/hub.ts) — F10 #14/#15 insights MUST derive from the same helpers, never re-implement.</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Founder-approved mock v9 (2026-08-01)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>F7 Net worth — by-type grouping</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>All CASH-bucket kinds merge under ONE "Cash and cash equivalents" group header (CASH_GROUP_LABEL); rows keep their own names. Class list orders by liquidity: Cash → Bonds &amp; CDs → Stocks/ETFs → Alternatives → property.</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>B47 finding 14 + approved mocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>F1 Connect — provider</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SnapTrade remains the shipping provider. Founder evaluating Plaid vs SnapTrade vs Teller (pivot ON HOLD 2026-08-02); credit-card transaction import is a design-first candidate pending the provider decision.</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Founder provider review</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Banded sections adopted (founder 2026-08-04): UX design v1.2 + detailed-design changelog + PRD amendment; SectionBand component + bandLight token; Home (4 bands) + Plan hub (6 bands) converted; 4 pins; 1400 green
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/FCC-core-55-70/FCC-core-PRD-v1.1-2026-07-01.xlsx
+++ b/docs/FCC-core-55-70/FCC-core-PRD-v1.1-2026-07-01.xlsx
@@ -841,7 +841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" style="24" min="1" max="1"/>
@@ -979,6 +979,28 @@
       <c r="D6" t="inlineStr">
         <is>
           <t>Founder provider review</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Asset classification (F1)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>AMENDMENT (founder 2026-08-04): cash = cash ONLY (checking/savings/HYSA/cash-mgmt/sweep). Money-market FUNDS class as Stocks/ETFs (dividend-paying funds, measured); CDs and T-bills class as Bonds &amp; CDs regardless of maturity (interest-paying, measured). Supersedes: money-market=cash (2026-07-19 live-verify mapping) and the build-34 #8 12-month CD split. Rationale: instruments that pay dividends/interest must live inside the Performance-measured buckets or earned-income and return calculations are silently wrong. Broker cash-sleeve dedupe unchanged (keyed on the cash_equivalent flag, not class).</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>BUILT 2026-08-04 (sync/import/capture/kind-map/glossary + engine: CD interest = balance × stated rate); 20+ pins rewritten; suite 1,396 green.</t>
         </is>
       </c>
     </row>

</xml_diff>